<commit_message>
sheet-sync cards: map list defines the maps; forfeits, half-edited cards, Self-Check SUM row, picture evidence
First real-sheet inventory: 575 cards, 2080 maps, 16/21 Self-Check rows
agree. The rest are explained by 'Map Forfeit' rows, cards whose panels are
filled before their map list, and in-progress series. A map panel now
counts only when it names its map; only map-list rows are maps; forfeited
and half-edited cards are counted, not imported. Unnamed pictures beside
ban text are reported as evidence for a reviewed alias, never applied.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Tjki2qjrj7kic2eZge7tfG
</commit_message>
<xml_diff>
--- a/pipeline/fixtures/gsheet/owcs_cards_fixture.xlsx
+++ b/pipeline/fixtures/gsheet/owcs_cards_fixture.xlsx
@@ -5377,6 +5377,731 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="51" name="Image 51" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="52" name="Image 52" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="53" name="Image 53" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="54" name="Image 54" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>58</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="55" name="Image 55" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>58</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="56" name="Image 56" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="57" name="Image 57" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="58" name="Image 58" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="59" name="Image 59" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="60" name="Image 60" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId60"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>20</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="61" name="Image 61" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId61"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>20</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="62" name="Image 62" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId62"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>23</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="63" name="Image 63" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>23</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="64" name="Image 64" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>54</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="65" name="Image 65" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>55</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="66" name="Image 66" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="67" name="Image 67" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="68" name="Image 68" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="69" name="Image 69" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>16</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="70" name="Image 70" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>20</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="71" name="Image 71" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>20</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="72" name="Image 72" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>23</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="73" name="Image 73" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>23</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="74" name="Image 74" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>76</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="75" name="Image 75" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>26</col>
+      <colOff>0</colOff>
+      <row>72</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="76" name="Image 76" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>23</col>
+      <colOff>0</colOff>
+      <row>59</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="77" name="Image 77" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>60</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="78" name="Image 78" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>13</col>
+      <colOff>0</colOff>
+      <row>65</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="152400" cy="152400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="79" name="Image 79" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -7156,7 +7881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C3:AS25"/>
+  <dimension ref="C3:AS77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="3">
@@ -7470,10 +8195,234 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>OWCS Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Round Robin [Bo3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Week 1 | Day 1 | Game 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FXG</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>FXE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>►</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Map Forfeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>►</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Map Forfeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="41"/>
+    <row r="55">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OWCS Japan</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Delta-1</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Delta-2</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Delta-3</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>Delta-4</t>
+        </is>
+      </c>
+      <c r="AB55" t="inlineStr">
+        <is>
+          <t>Delta-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Round Robin [Bo3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Week 1 | Day 2 | Game 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Fixture Delta [0-0]</t>
+        </is>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>Busan</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>FXD</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>FXE</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>FXD Ban</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>◄</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>►</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>FXE Ban</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="X68" t="inlineStr">
+        <is>
+          <t>Fixture Delta Wins!</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Mercy</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Juno</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Fixture Epsilon [0-0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="X71" t="inlineStr">
+        <is>
+          <t>Map: 2-1</t>
+        </is>
+      </c>
+      <c r="AA71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Series: </t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Gamma-1</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Gamma-2</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Gamma-3</t>
+        </is>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>Gamma-4</t>
+        </is>
+      </c>
+      <c r="AB77" t="inlineStr">
+        <is>
+          <t>Gamma-5</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="F12:I13"/>
     <mergeCell ref="F14:I15"/>
+    <mergeCell ref="F38:I39"/>
+    <mergeCell ref="F40:I41"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>